<commit_message>
updated scheme, scheme mapping and person upload endpoint
</commit_message>
<xml_diff>
--- a/backend/scheme-service/examples/scheme-mapping-upload-test.xlsx
+++ b/backend/scheme-service/examples/scheme-mapping-upload-test.xlsx
@@ -413,90 +413,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>scheme_id</t>
+          <t>state_scheme_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>parent_lgd_id</t>
+          <t>village_lgd_code</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>parent_lgd_level</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>parent_department_id</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>parent_department_level</t>
+          <t>sub_division_name</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>501</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1001</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>division</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SS-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>VLG-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Bengaluru North</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>502</v>
-      </c>
-      <c r="C3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1002</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>division</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SS-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VLG-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mysuru South</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>503</v>
-      </c>
-      <c r="C4" t="n">
-        <v>7</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1003</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>division</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SS-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>VLG-003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Invalid Subdivision</t>
         </is>
       </c>
     </row>

</xml_diff>